<commit_message>
Recette QA : consigner les résultats du cycle 1 dans le classeur
4 défauts clos (avec requalifications : DEF-003 mineur→majeur, DEF-001
mobile uniquement, DEF-002 requalifié). 3 demandes livrées. CR-001 laissé
en TRIAGED avec la raison : les chaînes t() sont les CLÉS de traduction.
Cycle 1 consigné : GO.

Ajout : e2e/diag.production.mjs — vérification indépendante sur le site RÉEL.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
+++ b/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
@@ -36,7 +36,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,13 @@
       <color rgb="007A8194"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000B6B2F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +110,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F3F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -188,6 +198,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -20589,9 +20602,9 @@
         </is>
       </c>
       <c r="T3" s="16" t="inlineStr"/>
-      <c r="U3" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
+      <c r="U3" s="21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="V3" s="16" t="inlineStr">
@@ -20599,12 +20612,20 @@
           <t>Othman</t>
         </is>
       </c>
-      <c r="W3" s="16" t="inlineStr"/>
-      <c r="X3" s="16" t="inlineStr"/>
+      <c r="W3" s="16" t="inlineStr">
+        <is>
+          <t>42601e8</t>
+        </is>
+      </c>
+      <c r="X3" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="Y3" s="16" t="inlineStr"/>
       <c r="Z3" s="16" t="inlineStr">
         <is>
-          <t>Reported as 'page design is terrible and size page not fit the browser page'. Split from the design rework, which is tracked as CR-011.</t>
+          <t>Majeur → confirmé MOBILE UNIQUEMENT. Aucun débordement sur ordinateur (1280/1366/1440/1920 = 0). Cause : halo décoratif de 440px sans overflow-hidden. Le grief « ne rentre pas » sur grand écran est un sujet de DESIGN, suivi en CR-011.</t>
         </is>
       </c>
     </row>
@@ -20707,9 +20728,9 @@
         </is>
       </c>
       <c r="T4" s="16" t="inlineStr"/>
-      <c r="U4" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
+      <c r="U4" s="21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="V4" s="16" t="inlineStr">
@@ -20717,12 +20738,20 @@
           <t>Othman</t>
         </is>
       </c>
-      <c r="W4" s="16" t="inlineStr"/>
-      <c r="X4" s="16" t="inlineStr"/>
+      <c r="W4" s="16" t="inlineStr">
+        <is>
+          <t>42601e8</t>
+        </is>
+      </c>
+      <c r="X4" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="Y4" s="16" t="inlineStr"/>
       <c r="Z4" s="16" t="inlineStr">
         <is>
-          <t>List the exact elements in the Test Log before fixing. e2e/outil.audit-clics.mjs already detects dead buttons — run it first to get the full list.</t>
+          <t>Requalifié. Aucun élément TROMPEUR sur les 7 tableaux de bord. Réel : 3 chiffres de la console plateforme sans `to` ni `onClick` → rendus en &lt;div&gt; inerte. Les 4 mènent désormais à #/app/schools (vérifié en production).</t>
         </is>
       </c>
     </row>
@@ -20824,9 +20853,9 @@
         </is>
       </c>
       <c r="T5" s="16" t="inlineStr"/>
-      <c r="U5" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
+      <c r="U5" s="21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="V5" s="16" t="inlineStr">
@@ -20834,12 +20863,20 @@
           <t>Othman</t>
         </is>
       </c>
-      <c r="W5" s="16" t="inlineStr"/>
-      <c r="X5" s="16" t="inlineStr"/>
+      <c r="W5" s="16" t="inlineStr">
+        <is>
+          <t>42601e8</t>
+        </is>
+      </c>
+      <c r="X5" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="Y5" s="16" t="inlineStr"/>
       <c r="Z5" s="16" t="inlineStr">
         <is>
-          <t>This is the defect half of note 6. Turning the one-pager into real routed pages is a separate product decision, tracked as CR-006.</t>
+          <t>Requalifié MINEUR → MAJEUR. Les liens ne « défilaient » pas : ils ne faisaient RIEN. Incompatibilité &lt;a href=#ancre&gt; / HashRouter — 9 liens morts. Corrigé + état actif ajouté. Vérifié en production : 0 → 1979.</t>
         </is>
       </c>
     </row>
@@ -20941,9 +20978,9 @@
         </is>
       </c>
       <c r="T6" s="16" t="inlineStr"/>
-      <c r="U6" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
+      <c r="U6" s="21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="V6" s="16" t="inlineStr">
@@ -20951,12 +20988,20 @@
           <t>Othman</t>
         </is>
       </c>
-      <c r="W6" s="16" t="inlineStr"/>
-      <c r="X6" s="16" t="inlineStr"/>
+      <c r="W6" s="16" t="inlineStr">
+        <is>
+          <t>42601e8</t>
+        </is>
+      </c>
+      <c r="X6" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="Y6" s="16" t="inlineStr"/>
       <c r="Z6" s="16" t="inlineStr">
         <is>
-          <t>Check at several widths — likely a flex alignment issue, so it may only show at some breakpoints.</t>
+          <t>Confirmé. Cause : la ligne de base d'un conteneur flex vient de son premier élément ; ici une icône SVG, sans ligne de base. Icône passée en inline.</t>
         </is>
       </c>
     </row>
@@ -32272,7 +32317,7 @@
       </c>
       <c r="O3" s="16" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>TRIAGED</t>
         </is>
       </c>
       <c r="P3" s="16" t="inlineStr"/>
@@ -32283,7 +32328,11 @@
         </is>
       </c>
       <c r="S3" s="16" t="inlineStr"/>
-      <c r="T3" s="16" t="inlineStr"/>
+      <c r="T3" s="16" t="inlineStr">
+        <is>
+          <t>PAS un remplacer-tout. 1108 occurrences : 457 en commentaires (à laisser), 49 dans t() — où la chaîne FRANÇAISE est la CLÉ de traduction : la modifier casse l'arabe en silence, sans qu'aucun test n'échoue. Il faut modifier l'appel ET la clé i18n.js dans le même geste, et choisir au cas par cas (· ici, virgule là). ~600 décisions : mérite une passe dédiée.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="108" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
@@ -32772,12 +32821,16 @@
           <t>S</t>
         </is>
       </c>
-      <c r="O9" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="P9" s="16" t="inlineStr"/>
+      <c r="O9" s="21" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P9" s="16" t="inlineStr">
+        <is>
+          <t>42601e8 · 2026-07-22</t>
+        </is>
+      </c>
       <c r="Q9" s="16" t="inlineStr"/>
       <c r="R9" s="16" t="inlineStr">
         <is>
@@ -32785,7 +32838,11 @@
         </is>
       </c>
       <c r="S9" s="16" t="inlineStr"/>
-      <c r="T9" s="16" t="inlineStr"/>
+      <c r="T9" s="16" t="inlineStr">
+        <is>
+          <t>Formulaire élargi (max-w-2xl → max-w-4xl). Vérifié : toujours 0 débordement à 390px.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="108" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
@@ -33121,7 +33178,11 @@
           <t>DEF-001</t>
         </is>
       </c>
-      <c r="T13" s="16" t="inlineStr"/>
+      <c r="T13" s="16" t="inlineStr">
+        <is>
+          <t>Porte désormais AUSSI le grief « la page ne rentre pas » sur grand écran : la mesure montre 0 débordement sur ordinateur, donc c'est du design, pas un défaut. Le débordement mobile réel a été corrigé (DEF-001, clos).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="108" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
@@ -33274,12 +33335,16 @@
           <t>M</t>
         </is>
       </c>
-      <c r="O15" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="P15" s="16" t="inlineStr"/>
+      <c r="O15" s="21" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P15" s="16" t="inlineStr">
+        <is>
+          <t>42601e8 · 2026-07-22</t>
+        </is>
+      </c>
       <c r="Q15" s="16" t="inlineStr"/>
       <c r="R15" s="16" t="inlineStr">
         <is>
@@ -33287,7 +33352,11 @@
         </is>
       </c>
       <c r="S15" s="16" t="inlineStr"/>
-      <c r="T15" s="16" t="inlineStr"/>
+      <c r="T15" s="16" t="inlineStr">
+        <is>
+          <t>Livré. Serveur : /api/forgot + /api/reset, jeton usage unique 60 min, réponse neutre, 5 demandes/h/IP, compte désactivé ignoré, sessions fermées à la réinitialisation. Web : #/mot-de-passe-oublie + #/reinitialiser + lien sur /login. Mode démo : la demande part à support@kogiagroup.com. 4 tests serveur + 10 vérif. navigateur.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="108" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
@@ -33440,12 +33509,16 @@
           <t>XS</t>
         </is>
       </c>
-      <c r="O17" s="16" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="P17" s="16" t="inlineStr"/>
+      <c r="O17" s="21" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P17" s="16" t="inlineStr">
+        <is>
+          <t>42601e8 · 2026-07-22</t>
+        </is>
+      </c>
       <c r="Q17" s="16" t="inlineStr"/>
       <c r="R17" s="16" t="inlineStr">
         <is>
@@ -33453,7 +33526,11 @@
         </is>
       </c>
       <c r="S17" s="16" t="inlineStr"/>
-      <c r="T17" s="16" t="inlineStr"/>
+      <c r="T17" s="16" t="inlineStr">
+        <is>
+          <t>Chip météo en une seule ligne (icône 20px + température) ; libellé et détail dans le panneau.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="108" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
@@ -39390,27 +39467,77 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="n"/>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
-      <c r="J3" s="16" t="n"/>
-      <c r="K3" s="16" t="n"/>
+    <row r="3" ht="64" customHeight="1">
+      <c r="A3" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Recette QA initiale</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>42601e8</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>Othman + Claude</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Pages publiques (accueil, connexion, pré-inscription) × 6 tailles ; tableaux de bord × 7 rôles ; parcours mot de passe oublié ; suites automatisées complètes.</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="I3" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="J3" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="L3" s="18">
         <f>IF(N(H3)=0,"",I3/H3)</f>
         <v/>
       </c>
-      <c r="M3" s="16" t="n"/>
-      <c r="N3" s="16" t="n"/>
-      <c r="O3" s="16" t="n"/>
-      <c r="P3" s="16" t="n"/>
-      <c r="Q3" s="16" t="n"/>
+      <c r="M3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="21" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="P3" s="16" t="inlineStr">
+        <is>
+          <t>Othman</t>
+        </is>
+      </c>
+      <c r="Q3" s="16" t="inlineStr">
+        <is>
+          <t>4 défauts trouvés et corrigés le jour même. 3 demandes livrées. core 54/54 · serveur 15/15 · e2e 131/131 · CI verte · vérifié sur le site réel.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="n"/>

</xml_diff>

<commit_message>
Épics ERP : plan séquencé (CR-017/018/021) + classeur QA à jour
docs/quality/erp-epics-plan.md — plan à décider avec Othman pour les 3 épics XL :
  · ce qui est DÉJÀ construit (refs.js = générateur unique + Luhn ; {idType,cin}
    par pays ; départements CR-019 ; modèle de rôles) — on ne le refait pas
  · CR-017 (référence partout, sans trou, affichée) : 1–1,5 sem, faible risque → 1er
  · CR-018 (entité Personne, N rôles) : 2–3 sem, risque élevé → après un 2e marché
  · CR-021 = définition « vrai ERP » qui chapeaute
  · 3 décisions à trancher : D-1 portée pour la vente, D-2 Person avant pilote ?,
    D-3 partie double ? Rien n'est lancé.

Classeur QA : CR-001, CR-006, CR-012 → DONE ; CR-011 annoté (3 directions
livrées, en attente du choix) ; CR-017/018/021 pointent vers le plan.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
+++ b/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
@@ -32343,10 +32343,14 @@
       </c>
       <c r="O3" s="16" t="inlineStr">
         <is>
-          <t>TRIAGED</t>
-        </is>
-      </c>
-      <c r="P3" s="16" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P3" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="Q3" s="16" t="inlineStr"/>
       <c r="R3" s="16" t="inlineStr">
         <is>
@@ -32356,7 +32360,7 @@
       <c r="S3" s="16" t="inlineStr"/>
       <c r="T3" s="16" t="inlineStr">
         <is>
-          <t>PAS un remplacer-tout. 1108 occurrences : 457 en commentaires (à laisser), 49 dans t() — où la chaîne FRANÇAISE est la CLÉ de traduction : la modifier casse l'arabe en silence, sans qu'aucun test n'échoue. Il faut modifier l'appel ET la clé i18n.js dans le même geste, et choisir au cas par cas (· ici, virgule là). ~600 décisions : mérite une passe dédiée.</t>
+          <t>LIVRÉ 2026-07-23. La passe de contenu (commit affa9ed) avait retiré 535 tirets du FR+AR ; il restait 3 tirets dans des chaînes RÉELLEMENT affichées : opsprofile.js (mode client) et 2 libellés d'autorité (locales.js BH/QA). Nettoyés (· et virgule). Recherche exhaustive : plus AUCUN tiret cadratin dans une chaîne rendue — il n'en reste que dans les commentaires de code (volontairement laissés). Critère d'acceptation atteint.</t>
         </is>
       </c>
     </row>
@@ -32794,10 +32798,14 @@
       </c>
       <c r="O8" s="22" t="inlineStr">
         <is>
-          <t>TRIAGED</t>
-        </is>
-      </c>
-      <c r="P8" s="16" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P8" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="Q8" s="16" t="inlineStr"/>
       <c r="R8" s="16" t="inlineStr">
         <is>
@@ -32811,7 +32819,7 @@
       </c>
       <c r="T8" s="16" t="inlineStr">
         <is>
-          <t>Le défaut « rien ne change au clic » est corrigé (DEF-003 : les ancres défilent + état actif). Des PAGES routées séparées avec URL propres restent un chantier plus large (SEO), à décider.</t>
+          <t>LIVRÉ 2026-07-23. La vitrine n'est plus une page unique à défilement : Accueil / Modules / Vos données / Tarifs / FAQ sont de VRAIES routes (#/, #/modules, #/donnees, #/tarifs, #/faq) sous une coquille partagée (app/src/pages/site/). URL propre partageable, bouton précédent respecté, entrée active marquée, accès direct à chaque page. Vérifié au navigateur (13/13) + e2e complet vert. Landing.jsx laissé en place, non importé.</t>
         </is>
       </c>
     </row>
@@ -33266,7 +33274,7 @@
       </c>
       <c r="T13" s="16" t="inlineStr">
         <is>
-          <t>Le débordement mobile réel est corrigé (DEF-001). La refonte visuelle complète de l’écran de connexion reste un choix de design d’Othman.</t>
+          <t>En attente du CHOIX d'Othman. 3 directions rendues et comparables (artefact « Coreon EDU · Connexion — 3 directions ») : 01 Cinématique (sombre, l'actuelle raffinée), 02 Clair éditorial (recommandée, alignée sur le site clair validé), 03 Focus (carte centrée minimale). La nouvelle accroche (CR-012) est déjà dans les trois. Dès qu'il choisit un numéro → câblage dans Login.jsx.</t>
         </is>
       </c>
     </row>
@@ -33340,10 +33348,14 @@
       </c>
       <c r="O14" s="22" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
-        </is>
-      </c>
-      <c r="P14" s="16" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P14" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="Q14" s="16" t="inlineStr"/>
       <c r="R14" s="16" t="inlineStr">
         <is>
@@ -33353,7 +33365,7 @@
       <c r="S14" s="16" t="inlineStr"/>
       <c r="T14" s="16" t="inlineStr">
         <is>
-          <t>Mention « Tunisie » retirée de l’écran de connexion. La réécriture des accroches marketing relève d’un choix éditorial.</t>
+          <t>LIVRÉ 2026-07-23. Accroche de connexion réécrite (les lignes qu'Othman jugeait peu attractives) : « Toute votre école, sur une seule plateforme. » + sous-titre admissions/évaluation/finances/communication. Ton international, plus « pas un ERP de plus ». FR + AR (i18n.js) dans le même geste. La refonte VISUELLE (couleurs/mise en page) relève de CR-011.</t>
         </is>
       </c>
     </row>
@@ -33804,7 +33816,7 @@
       <c r="S19" s="16" t="inlineStr"/>
       <c r="T19" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPÉCIFIÉ (plus bloqué par la recherche) : voir docs/quality/role-model.md §7 pour le backlog concret. Reste un chantier de plusieurs semaines qui touche le modèle de données — à planifier avec Othman. </t>
+          <t>SPÉCIFIÉ (plus bloqué par la recherche) : voir docs/quality/role-model.md §7 pour le backlog concret. Reste un chantier de plusieurs semaines qui touche le modèle de données — à planifier avec Othman.   |  PLAN 2026-07-23 : docs/quality/erp-epics-plan.md — séquencement (CR-017 d'abord, faible risque ; CR-018 après un 2ᵉ marché) + 3 décisions à prendre (D-1 portée « vrai ERP », D-2 Person avant pilote ?, D-3 partie double ?). Rien n'est lancé : attend la décision d'Othman.</t>
         </is>
       </c>
     </row>
@@ -33891,7 +33903,7 @@
       <c r="S20" s="16" t="inlineStr"/>
       <c r="T20" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPÉCIFIÉ (plus bloqué par la recherche) : voir docs/quality/role-model.md §7 pour le backlog concret. Reste un chantier de plusieurs semaines qui touche le modèle de données — à planifier avec Othman. </t>
+          <t>SPÉCIFIÉ (plus bloqué par la recherche) : voir docs/quality/role-model.md §7 pour le backlog concret. Reste un chantier de plusieurs semaines qui touche le modèle de données — à planifier avec Othman.   |  PLAN 2026-07-23 : docs/quality/erp-epics-plan.md — séquencement (CR-017 d'abord, faible risque ; CR-018 après un 2ᵉ marché) + 3 décisions à prendre (D-1 portée « vrai ERP », D-2 Person avant pilote ?, D-3 partie double ?). Rien n'est lancé : attend la décision d'Othman.</t>
         </is>
       </c>
     </row>
@@ -34160,7 +34172,7 @@
       <c r="S23" s="16" t="inlineStr"/>
       <c r="T23" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPÉCIFIÉ (plus bloqué par la recherche) : voir docs/quality/role-model.md §7 pour le backlog concret. Reste un chantier de plusieurs semaines qui touche le modèle de données — à planifier avec Othman. </t>
+          <t>SPÉCIFIÉ (plus bloqué par la recherche) : voir docs/quality/role-model.md §7 pour le backlog concret. Reste un chantier de plusieurs semaines qui touche le modèle de données — à planifier avec Othman.   |  PLAN 2026-07-23 : docs/quality/erp-epics-plan.md — séquencement (CR-017 d'abord, faible risque ; CR-018 après un 2ᵉ marché) + 3 décisions à prendre (D-1 portée « vrai ERP », D-2 Person avant pilote ?, D-3 partie double ?). Rien n'est lancé : attend la décision d'Othman.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CR-011 : refonte de l'écran de connexion — direction « Clair éditorial »
Choisie parmi 3 directions rendues (Othman, 2026-07-23). L'écran de connexion
quitte le sombre cinématique pour un parti pris CLAIR, aligné sur kogiagroup.com
(le site clair validé) : il dit « école », pas « banque ».

  · formulaire à gauche sur un dégradé lavande (blanc → #F3F0FF)
  · panneau marque à droite (clair) montrant la VRAIE maquette produit —
    l'évaluation en direct (composant EvalMock réutilisé depuis site/shared.jsx)
  · nouvelle accroche CR-012 intégrée ; violet Coreon en accent, cyan décor only
  · logo en haut seulement, 0 débordement à 390px, mouvement coupé si réduit

Vérifié : 10/10 au navigateur (champs, pastilles démo → tableau de bord, mobile
390px sans débordement, 0 erreur console). DEF-001 (débordement) déjà clos.
Classeur QA : CR-011 → DONE.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
+++ b/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
@@ -33257,10 +33257,14 @@
       </c>
       <c r="O13" s="22" t="inlineStr">
         <is>
-          <t>TRIAGED</t>
-        </is>
-      </c>
-      <c r="P13" s="16" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="P13" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="Q13" s="16" t="inlineStr"/>
       <c r="R13" s="16" t="inlineStr">
         <is>
@@ -33274,7 +33278,7 @@
       </c>
       <c r="T13" s="16" t="inlineStr">
         <is>
-          <t>En attente du CHOIX d'Othman. 3 directions rendues et comparables (artefact « Coreon EDU · Connexion — 3 directions ») : 01 Cinématique (sombre, l'actuelle raffinée), 02 Clair éditorial (recommandée, alignée sur le site clair validé), 03 Focus (carte centrée minimale). La nouvelle accroche (CR-012) est déjà dans les trois. Dès qu'il choisit un numéro → câblage dans Login.jsx.</t>
+          <t>LIVRÉ 2026-07-23. Refonte de l'écran de connexion, direction « Clair éditorial » (choisie parmi 3 directions rendues) : fond clair aligné sur le site validé, formulaire à gauche, panneau marque à droite montrant la maquette produit en direct (évaluation). Violet Coreon en accent, logo en haut seulement, 0 débordement à 390px, mouvement coupé si réduit. Nouvelle accroche (CR-012) intégrée. Vérifié : 10/10 navigateur + suite e2e. DEF-001 déjà clos.</t>
         </is>
       </c>
     </row>

</xml_diff>